<commit_message>
updating the script for some quality of life features
</commit_message>
<xml_diff>
--- a/tools/input/products.xlsx
+++ b/tools/input/products.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>name</t>
   </si>
@@ -24,55 +24,43 @@
     <t>price</t>
   </si>
   <si>
-    <t>image</t>
-  </si>
-  <si>
     <t>description</t>
   </si>
   <si>
     <t>Laptop Pro</t>
   </si>
   <si>
-    <t>laptop.jpg</t>
-  </si>
-  <si>
-    <t>High performance laptop</t>
-  </si>
-  <si>
-    <t>iPhone 14</t>
-  </si>
-  <si>
-    <t>iphone.jpg</t>
-  </si>
-  <si>
-    <t>Latest Apple phone</t>
-  </si>
-  <si>
-    <t>Headphones</t>
-  </si>
-  <si>
-    <t>headphones.jpg</t>
-  </si>
-  <si>
-    <t>Noise cancelling headset</t>
-  </si>
-  <si>
-    <t>Smart Watch</t>
-  </si>
-  <si>
-    <t>watch.jpg</t>
-  </si>
-  <si>
-    <t>Fitness tracking watch</t>
-  </si>
-  <si>
-    <t>Tablet S</t>
-  </si>
-  <si>
-    <t>tablet.jpg</t>
-  </si>
-  <si>
-    <t>Lightweight tablet</t>
+    <t>High performance laptop built for demanding workflows and all-day productivity.</t>
+  </si>
+  <si>
+    <t>Wireless Headphones</t>
+  </si>
+  <si>
+    <t>Premium over-ear headphones with active noise cancellation and rich, balanced sound.</t>
+  </si>
+  <si>
+    <t>Smartphone X</t>
+  </si>
+  <si>
+    <t>Edge-to-edge display, powerful camera system, and a battery that lasts all day.</t>
+  </si>
+  <si>
+    <t>Smartwatch Series 5</t>
+  </si>
+  <si>
+    <t>Track fitness, notifications, and health metrics from your wrist with style.</t>
+  </si>
+  <si>
+    <t>Mechanical Keyboard</t>
+  </si>
+  <si>
+    <t>Compact mechanical keyboard with tactile switches for a precise typing experience.</t>
+  </si>
+  <si>
+    <t>4K Monitor</t>
+  </si>
+  <si>
+    <t>Crisp 4K resolution on a slim, color-accurate panel perfect for work and play.</t>
   </si>
 </sst>
 </file>
@@ -425,8 +413,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.28515625" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" customWidth="1"/>
+    <col min="3" max="3" width="63.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -438,78 +431,77 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" spans="1:4" ht="111.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
       </c>
       <c r="B2" s="2">
         <v>1200</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:4" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="B3" s="2">
+        <v>240</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="1:4" ht="81.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="2">
-        <v>900</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="B4" s="2">
+        <v>899</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D4" s="2"/>
+    </row>
+    <row r="5" spans="1:4" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="B5" s="2">
+        <v>320</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="2">
-        <v>150</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" spans="1:4" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="B6" s="2">
+        <v>130</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" spans="1:4" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="2">
-        <v>200</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="B7" s="2">
+        <v>560</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="2">
-        <v>400</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>